<commit_message>
feat: complete content readiness and NPC autonomy follow-up
Require autonomous cultivators to reach authored cushions and let exhausted residents return to assigned beds. Include personal life, combat AI, retreat, direct-vassal storage access, content authoring repairs, and current documentation.
</commit_message>
<xml_diff>
--- a/docs/40-process/273-current-art-asset-register.xlsx
+++ b/docs/40-process/273-current-art-asset-register.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术清单" sheetId="1" r:id="Rc69a64c56f72451d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工程明细" sheetId="2" r:id="R7a58fddd3355417b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="美术清单" sheetId="1" r:id="Reb2f4ff963d24405"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工程明细" sheetId="2" r:id="R896f676bf06147cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -508,7 +508,7 @@
         <x:v>导出时间 UTC</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>UTC 2026-10-21T02:35:41.976Z</x:v>
+        <x:v>UTC 2026-10-21T07:44:07.340Z</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
       <x:c r="D4" s="3"/>
@@ -523,7 +523,7 @@
         <x:v>源 SHA-256</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>7948558a744f21284a04355c0351ed4fcf7745fef2da6ea946bc827eca422ab1</x:v>
+        <x:v>75f825b8e4fcd59d5dd847b1839f58c2942df060ed8617f94a528c283d27a42e</x:v>
       </x:c>
       <x:c r="C5" s="3"/>
       <x:c r="D5" s="3"/>
@@ -2208,7 +2208,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra69bf79992bc4114"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R638cf37beb0c4bd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2322,7 +2322,7 @@
         <x:v>导出时间 UTC</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>UTC 2026-10-21T02:35:41.976Z</x:v>
+        <x:v>UTC 2026-10-21T07:44:07.340Z</x:v>
       </x:c>
       <x:c r="C4" s="3"/>
       <x:c r="D4" s="3"/>
@@ -2349,7 +2349,7 @@
         <x:v>源 SHA-256</x:v>
       </x:c>
       <x:c r="B5" s="2" t="str">
-        <x:v>7948558a744f21284a04355c0351ed4fcf7745fef2da6ea946bc827eca422ab1</x:v>
+        <x:v>75f825b8e4fcd59d5dd847b1839f58c2942df060ed8617f94a528c283d27a42e</x:v>
       </x:c>
       <x:c r="C5" s="3"/>
       <x:c r="D5" s="3"/>
@@ -2536,7 +2536,7 @@
         <x:v>Assets/Scripts/Unity/Host/HostSpriteFactory.cs；候选原图 ArtSource/Batches/Batch_20261016_01/Originals/ART-CHAR-001_common_villagers_3up_v01.png；候选新图 ArtSource/Batches/Batch_Codex_001/Originals/ART-CHAR-001_idle_4dir_1f_sheet_v01.png；ArtSource/Batches/Batch_Codex_001/Originals/ART-CHAR-001_walk_4dir_4f_sheet_v01.png；ArtSource/Batches/Batch_Codex_001/Originals/ART-CHAR-001_work_4dir_4f_sheet_v01.png；ArtSource/Batches/Batch_Codex_002/Sheets/ART-CHAR-001_walk_4dir_4f_sheet_v02.png；ArtSource/Batches/Batch_Codex_002/character_manifest.json；Step A Assets/Art/Characters/Resources/ART-CHAR-001_{idle,walk,work,attack}_v02.png；Batch_Codex_003/Frames/ART-CHAR-001_villager_sleep_v03.png；Assets/Art/Characters/Resources/ART-CHAR-001_villager_sleep_v03.png；部件原图 ArtSource/Batches/Batch_ModularRig_001/Originals/ART-CHAR-001_HumanCommonRig_parts_v01.png；样机运行图 Assets/Art/Characters/Resources/ART-CHAR-001_HumanCommonRig_parts_v01.png</x:v>
       </x:c>
       <x:c r="M9" s="11" t="str">
-        <x:v>EntityViewSpawner 的 SpriteRenderer；正式人物图集映射待确认；Step A EntityViewSpawner→EntityView；仅 base:character_ch01_ref_mortal_a 与 base:character_village_recruit 使用村民四方向图集；卧姿由 EntityView 读取真实 SleepPhase 与床位占用显示</x:v>
+        <x:v>EntityViewSpawner 的 SpriteRenderer；正式人物 DefinitionId→Profile 映射见 HostAppearanceMappings.json；Step A EntityViewSpawner→EntityView；仅 base:character_ch01_ref_mortal_a 与 base:character_village_recruit 使用村民四方向图集；卧姿由 EntityView 读取真实 SleepPhase 与床位占用显示</x:v>
       </x:c>
       <x:c r="N9" s="11" t="str">
         <x:v>未验收</x:v>
@@ -2666,7 +2666,7 @@
         <x:v>Assets/Art/Characters/NPCs/Supervisor/CHR_NPC_Supervisor_Idle_Down.png；候选原图 ArtSource/Batches/Batch_20261016_01/Originals/ART-CHAR-003_supervisor_v01.png；ArtSource/Batches/Batch_Codex_002/Static/ART-CHAR-003_supervisor_idle_south_v02.png；ArtSource/Batches/Batch_Codex_003/Frames/ART-CHAR-003_supervisor_sleep_v03.png；Assets/Art/Characters/Resources 对应卧姿；部件原图 ArtSource/Batches/Batch_ModularRig_002/Originals/ART-CHAR-002_003_005_HumanCommonRig_sideheads_v01.png；部件原图 ArtSource/Batches/Batch_ModularRig_002/Originals/ART-CHAR-003_supervisor_HumanCommonRig_parts_v01.png</x:v>
       </x:c>
       <x:c r="M11" s="11" t="str">
-        <x:v>Supervisor.prefab 有引用；正式人物映射待确认；本轮 EntityView主管身份南向静图；Assets/Art/Characters/Resources</x:v>
+        <x:v>Supervisor.prefab 有引用；正式人物与主管 Rig 映射见 HostAppearanceMappings.json；本轮 EntityView主管身份南向静图；Assets/Art/Characters/Resources</x:v>
       </x:c>
       <x:c r="N11" s="11" t="str">
         <x:v>未验收</x:v>
@@ -2731,7 +2731,7 @@
         <x:v>Assets/Art/Characters/NPCs/Guard/CHR_NPC_Guard_Idle_Down.png；候选原图 ArtSource/Batches/Batch_20261016_01/Originals/ART-CHAR-004_patrol_guard_v01.png；候选新图 ArtSource/Batches/Batch_Codex_001/Originals/ART-CHAR-004_idle_4dir_1f_sheet_v01.png；ArtSource/Batches/Batch_Codex_001/Originals/ART-CHAR-004_walk_4dir_4f_sheet_v01.png；ArtSource/Batches/Batch_Codex_001/Originals/ART-CHAR-004_attack_4dir_4f_sheet_v01.png；ArtSource/Batches/Batch_Codex_002/Sheets/ART-CHAR-004_attack_4dir_4f_sheet_v02.png；Step A Assets/Art/Characters/Resources/ART-CHAR-004_{idle,walk,attack}_v02.png；ArtSource/Batches/Batch_Codex_003/Frames/ART-CHAR-004_guard_sleep_v03.png；Assets/Art/Characters/Resources 对应卧姿；部件原图 ArtSource/Batches/Batch_ModularRig_001/Originals/ART-CHAR-004_HumanCommonRig_parts_v01.png；样机运行图 Assets/Art/Characters/Resources/ART-CHAR-004_HumanCommonRig_parts_v01.png</x:v>
       </x:c>
       <x:c r="M12" s="11" t="str">
-        <x:v>Guard.prefab 有引用；正式人物映射待确认；Step A EntityViewSpawner→EntityView；guard_a/b/c 共用同一缓存图集</x:v>
+        <x:v>Guard.prefab 有引用；正式人物映射见 HostAppearanceMappings.json；Step A EntityViewSpawner→EntityView；guard_a/b/c 共用同一缓存图集</x:v>
       </x:c>
       <x:c r="N12" s="11" t="str">
         <x:v>未验收</x:v>
@@ -5006,13 +5006,13 @@
         <x:v>待确认；ArtSource/Batches/Batch_Codex_002/Previews/ART-UI-002_003_32px_readability_v02.png</x:v>
       </x:c>
       <x:c r="M47" s="11" t="str">
-        <x:v>ItemId到图标映射待确认；本轮 HostInventoryPanel五种现有ItemId背包格图标；Assets/Art/UI/Resources；HostGroundLootVisual 与 HostAppearanceMappings.json 读取图标及地面类别。</x:v>
+        <x:v>现有五种 ItemId 图标映射见 HostAppearanceMappings.json；本轮 HostInventoryPanel五种现有ItemId背包格图标；Assets/Art/UI/Resources；HostGroundLootVisual 与 HostAppearanceMappings.json 读取图标及地面类别。</x:v>
       </x:c>
       <x:c r="N47" s="11" t="str">
         <x:v>未验收</x:v>
       </x:c>
       <x:c r="O47" s="11" t="str">
-        <x:v>登记当前5个基本Item定义，不等于要5张独立原画；Batch_Codex_002：按当前 5 个 Item 定义制作图标并拆件；实际 ItemId 映射未接。；2026-10-16 本轮：仅上述实际运行范围接入，Unity PlayMode未验收。；313 地面功法书、斗技卷轴和药草/包裹轮廓已接线；最新洞府显示与拾取仍待窄范围现场复看。</x:v>
+        <x:v>登记当前5个基本Item定义，不等于要5张独立原画；Batch_Codex_002：按当前 5 个 Item 定义制作图标并拆件；实际 ItemId 映射已接，药草地面类别已显式配置。；2026-10-16 本轮：仅上述实际运行范围接入，Unity PlayMode未验收。；313 地面功法书、斗技卷轴和药草/包裹轮廓已接线；最新洞府显示与拾取仍待窄范围现场复看。</x:v>
       </x:c>
       <x:c r="P47" s="11" t="str">
         <x:v>5基础Item</x:v>
@@ -5266,13 +5266,13 @@
         <x:v>Assets/Scripts/Unity/Host/HostFactionFlagPresenter.cs；ArtSource/Batches/Batch_Codex_002/Static/ART-UI-007_interact_rune_v01.png</x:v>
       </x:c>
       <x:c r="M51" s="11" t="str">
-        <x:v>世界Sprite/文字overlay；正式标记映射待确认；本轮 HostMapGraybox 的正式地点标签叠加 site_marker 静态牌匾，文字仍动态，交互符文未接；Assets/Art/UI/Resources</x:v>
+        <x:v>世界Sprite/文字overlay；地点石牌已按307撤除，地点仍显示动态文字；交互符文未接；Assets/Art/UI/Resources</x:v>
       </x:c>
       <x:c r="N51" s="11" t="str">
         <x:v>未验收</x:v>
       </x:c>
       <x:c r="O51" s="11" t="str">
-        <x:v>名字、地点文字始终动态生成；正俯视世界标记可借修仙旗帜/石碑视觉语汇；石碑和法阵仍是待确认风格候选；Batch_Codex_002：交互符文与地点石牌新候选；旗帜复用 ROOM-008，动态文字不烘焙。；2026-10-16 本轮：地点牌匾已运行接线，独立旗帜/交互符文未接，Unity视觉待验。</x:v>
+        <x:v>名字、地点文字始终动态生成；正俯视世界标记可借修仙旗帜/石碑视觉语汇；石碑和法阵仍是待确认风格候选；Batch_Codex_002：交互符文与地点石牌新候选；旗帜复用 ROOM-008，动态文字不烘焙。；2026-10-16 地点牌匾曾接线；2026-10-20 按制作人截图从正式地点标签撤除。独立旗帜/交互符文未接，Unity视觉待验。</x:v>
       </x:c>
       <x:c r="P51" s="11" t="str">
         <x:v>12旗+22地点</x:v>
@@ -6086,7 +6086,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51aad0af31664fe8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43e02a88cc694133"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>